<commit_message>
feat(avance): plantilla 4 hojas + peso horas-hombre en hoja Avance
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/lib/services/excelAvanceGenerator/template/reporte-semanal-avance.template.xlsx
+++ b/src/lib/services/excelAvanceGenerator/template/reporte-semanal-avance.template.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
@@ -8,6 +8,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporte" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Avance" sheetId="3" r:id="rId14"/>
+    <sheet name="Curva S" sheetId="4" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Datos'!$A$1:$K$26</definedName>
@@ -37,7 +39,7 @@
     <numFmt numFmtId="178" formatCode="0.00000%"/>
     <numFmt numFmtId="179" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@"/>
   </numFmts>
-  <fonts count="53">
+  <fonts count="56">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -380,8 +382,26 @@
       <color theme="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -484,6 +504,30 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFA5000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF383838"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="96">
     <border>
@@ -1544,7 +1588,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13"/>
   </cellStyleXfs>
-  <cellXfs count="433">
+  <cellXfs count="442">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2642,6 +2686,19 @@
     <xf numFmtId="49" fontId="2" fillId="4" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="53" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="53" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7481,4 +7538,187 @@
     <brk id="64" min="0" max="15" man="1"/>
   </rowBreaks>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R50"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="7.7" customWidth="1"/>
+    <col min="2" max="2" width="52.3" customWidth="1"/>
+    <col min="3" max="3" width="13.6" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15.6" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5">
+      <c r="B5" s="433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proyecto:</t>
+        </is>
+      </c>
+      <c r="F5">
+        <f>+Datos!E7</f>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codido PEP</t>
+        </is>
+      </c>
+      <c r="F6">
+        <f>+Datos!E14</f>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OC:</t>
+        </is>
+      </c>
+      <c r="F7">
+        <f>+Datos!E13</f>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fecha de Inicio</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AÑO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="E10" s="434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEMANA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="E11" s="434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FECHA DE CORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pesos Globales</t>
+        </is>
+      </c>
+      <c r="D12" s="434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pesos Parciales</t>
+        </is>
+      </c>
+      <c r="E12" s="434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gbl LB1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="E13" s="434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gbl REAL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="F5:R5"/>
+    <mergeCell ref="F6:R6"/>
+    <mergeCell ref="F7:R7"/>
+    <mergeCell ref="B12:B13"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R40"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proyecto:</t>
+        </is>
+      </c>
+      <c r="C3">
+        <f>+Datos!E7</f>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codido PEP</t>
+        </is>
+      </c>
+      <c r="C4">
+        <f>+Datos!E14</f>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OC:</t>
+        </is>
+      </c>
+      <c r="C5">
+        <f>+Datos!E13</f>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEMANA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fecha de corte</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PREVISTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Variacion curva S</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>